<commit_message>
Add vault dashboard and attachment upload flows, expand AI meeting notes/summary test coverage
Introduces vault reports page object and dashboard spec, mobile upload-attachment
flows for iOS/Android, session state and attachment provisioning utilities, and
audio/xlsx test fixtures for AI meeting notes and conversation summary tests.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/playwright/testdata/summary-runs.xlsx
+++ b/playwright/testdata/summary-runs.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="4000" windowWidth="35840" windowHeight="16980"/>
+    <workbookView xWindow="0" yWindow="3940" windowWidth="35840" windowHeight="16980"/>
   </bookViews>
   <sheets>
     <sheet sheetId="1" name="Summaries" state="visible" r:id="rId4"/>
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
   <si>
     <t>Run Timestamp</t>
   </si>
@@ -98,6 +98,113 @@
   </si>
   <si>
     <t>nutriglow2: Invest more in the rise of large language models before AI outgrows our ability to manage it. nutriglow6: Prioritize the adoption of generative AI coding assistants as the highest-leverage move for AI. nutriglow10: Pilot AI-driven automated decision-making on a smaller scale before rolling it out further. nutriglow2: Pair STEM curriculum redesign with clear accountability measures so education doesn't drift off course. nutriglow6: Keep a close eye on student mental health support as a likely deciding factor for education. nutriglow10: Invest more in the affordability of higher education before education outgrows our ability to manage it.</t>
+  </si>
+  <si>
+    <t>2026-08-13T18:58:16.554Z</t>
+  </si>
+  <si>
+    <t>10 User High Volume Discussion 1786646011928</t>
+  </si>
+  <si>
+    <t>Summary: Aug 14, 2026 — The group discussed how the rise of large language models (LLMs) is reshaping artificial intelligence (AI), with nutriglow2 noting structural reforms are still needed, nutriglow9 raising oversight concerns, and nutriglow8 emphasizing LLMs touch nearly every part of AI systems. The adoption of generative AI coding assistants was debated; nutriglow7 called it the biggest recent shift in AI, while nutriglow9 pushed back, and nutriglow10 warned of over-reliance risks. AI-driven automated decision-making was discussed, with nutriglow10 suggesting it is currently overhyped but will matter more in five years, and nutriglow7 expressing concern it benefits only a few players. The push for AI regulation was noted as already reshaping AI faster than expected, with nutriglow8 warning regulation could outpace AI's ability to adapt. In education, the shortage of qualified teachers, STEM curriculum redesign, student mental health support, and affordability of higher education were all identified as key pressures, with nutriglow2 recommending pairing STEM redesign with clear accountability measures. Healthcare topics included health equity across income groups, strain on emergency departments, telemedicine adoption, and the shortage of primary care providers, with nutriglow10 suggesting piloting emergency department solutions at smaller scale first. Geopolitics discussion covered semiconductor supply chain tensions, the balance of power between major economies, the rise of regional security agreements, use of sanctions as a diplomatic tool, and energy dependence between nations. In politics, bipartisan policy negotiations, redistricting, the influence of lobbying groups, and transparency in government spending were debated, with nutriglow6 recommending pairing lobbying accountability with clear measures. Technology topics included cloud infrastructure adoption, data privacy regulation, the shift to edge computing, open-source software ecosystems, and developer productivity tooling. Economic discussions focused on small business access to credit, wage growth versus cost of living, the housing affordability crisis, and shifts in consumer spending. Climate topics included climate migration, EV adoption pace, the transition to renewable energy, and carbon pricing mechanisms. Cricket discussions covered player workload management, DRS and review technology, the red-ball vs. white-ball balance, and the emergence of talent from smaller cricketing nations. Basketball topics included the salary cap's impact on roster decisions, crowded schedules straining young players, the evolution of defensive schemes, and globalization of the sport's fanbase.</t>
+  </si>
+  <si>
+    <t>nutriglow2: Pair STEM curriculum redesign with clear accountability measures so education doesn't drift off course. nutriglow10: Pilot the strain on emergency departments on a smaller scale within healthcare before rolling it out further. nutriglow6: Prioritize the adoption of generative AI coding assistants as the highest-leverage move for AI. nutriglow10: Invest more in the affordability of higher education before education outgrows our ability to manage it. nutriglow10: Invest more in the shift in consumer spending before the economy outgrows our ability to manage it. nutriglow2: Pair wage growth versus cost of living with clear accountability measures so the economy doesn't drift off course. nutriglow6: Prioritize the use of sanctions as a diplomatic tool as the highest-leverage move for geopolitics. nutriglow6: Prioritize the transition to renewable energy given how much it affects climate.</t>
+  </si>
+  <si>
+    <t>2026-08-14T06:29:23.942Z</t>
+  </si>
+  <si>
+    <t>Bullet Format Test 1786688734</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary:
+• Aug 14, 2026 — nutriglow1 opened a discussion asking how the rise of large language models (LLMs) will change AI over the next few years.
+• nutriglow2 noted that LLMs will have real impact but that AI still needs structural reforms alongside them.
+• nutriglow5 offered a contrasting view, suggesting LLMs are not as central to AI as commonly assumed.
+• nutriglow6 warned that LLMs could backfire if AI isn't ready, while nutriglow9 raised concerns about insufficient oversight in LLM adoption.
+• nutriglow2 recommended investing more in LLMs before AI outgrows our ability to manage it, and nutriglow3 predicted LLMs will be a defining story in AI over the next decade.
+• nutriglow5 shifted the discussion to generative AI coding assistants, asking about their adoption within AI.
+• nutriglow7 called it the biggest recent shift in AI, while nutriglow9 pushed back, saying it hasn't made much difference. nutriglow10 cautioned against over-reliance.
+• nutriglow6 suggested prioritizing adoption of generative AI coding assistants as the highest-leverage move for AI.
+• nutriglow9 raised the topic of AI-driven automated decision-making, questioning whether it solves problems or adds complexity.
+• nutriglow10 called it currently overhyped but significant in five years. nutriglow4 warned it can widen gaps, and nutriglow7 expressed concern it benefits only a few players.
+• nutriglow10 proposed piloting AI-driven automated decision-making on a smaller scale before broader rollout.
+• nutriglow3 introduced the topic of AI regulation, with nutriglow4 noting it is already reshaping AI faster than most realize.
+• nutriglow8 cautioned that AI regulation could move faster than AI can adapt, while nutriglow10 noted the mechanics of regulation explain AI's rapid pace of change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. nutriglow2: Invest more in the rise of large language models before AI outgrows our ability to manage it.
+2. nutriglow6: Prioritize the adoption of generative AI coding assistants as the highest-leverage move for AI.
+3. nutriglow10: Pilot AI-driven automated decision-making on a smaller scale within AI before rolling it out further.</t>
+  </si>
+  <si>
+    <t>2026-08-14T06:39:28.223Z</t>
+  </si>
+  <si>
+    <t>Healthcare Topic Test 1786689350</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary:
+• Aug 14, 2026 — nutriglow1 opened the discussion by asking how telemedicine adoption will change healthcare over the next few years.
+• nutriglow2 noted telemedicine will have real impact but structural reforms are still needed alongside it.
+• nutriglow5 pushed back, suggesting telemedicine adoption is not as central to healthcare as commonly assumed, while nutriglow6 warned it could backfire if healthcare systems aren't ready.
+• nutriglow9 raised concern about telemedicine being adopted without sufficient oversight, and nutriglow10 noted it is already a major planning consideration for healthcare organizations.
+• nutriglow2 recommended investing more in telemedicine adoption before healthcare outgrows the ability to manage it.
+• nutriglow5 shifted the discussion to the shortage of primary care providers, which nutriglow7 called the biggest recent shift in healthcare and nutriglow4 identified as a top field priority.
+• nutriglow6 suggested prioritizing the primary care provider shortage as the highest-leverage move for healthcare improvement.
+• nutriglow9 raised whether the rising cost of prescription drugs is solving problems or adding complexity. nutriglow10 felt it is currently overhyped but will matter more in five years.
+• nutriglow7 expressed concern that rising prescription drug costs benefit only a few players, while nutriglow4 warned it could widen gaps in healthcare.
+• nutriglow10 proposed piloting prescription drug cost strategies on a smaller scale before broader rollout.
+• nutriglow3 introduced the rise of AI-assisted diagnostics, with nutriglow4 noting it is already reshaping healthcare faster than most realize.
+• nutriglow8 cautioned that AI-assisted diagnostics may advance faster than healthcare can adapt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. nutriglow2: Invest more in telemedicine adoption before healthcare outgrows our ability to manage it.
+2. nutriglow6: Prioritize addressing the shortage of primary care providers as the highest-leverage move for healthcare.
+3. nutriglow10: Pilot strategies around the rising cost of prescription drugs on a smaller scale within healthcare before rolling out further.</t>
+  </si>
+  <si>
+    <t>2026-08-14T07:27:59.713Z</t>
+  </si>
+  <si>
+    <t>Spotcheck Fix Test 1786692180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary:
+• Aug 14, 2026 — nutriglow1 opened a discussion asking how the rise of large language models (LLMs) will change AI over the next few years.
+• nutriglow2 noted that LLMs will have real impact but AI still needs structural reforms alongside them.
+• nutriglow5 pushed back, arguing LLMs are not as central to AI as commonly assumed, while nutriglow6 warned they could backfire without proper readiness.
+• nutriglow9 raised concern that LLMs could be adopted in AI without sufficient oversight, and nutriglow10 noted LLMs are already a major planning consideration for organizations.
+• nutriglow2 recommended investing more in LLMs before AI outgrows our ability to manage it, and nutriglow3 predicted LLMs will be one of the defining stories in AI over the next decade.
+• The group shifted to discussing generative AI coding assistants, with nutriglow7 calling their adoption the biggest recent shift in AI and nutriglow2 noting they address a core bottleneck.
+• nutriglow3 worried adoption of coding assistants may outpace necessary safeguards, and nutriglow6 suggested prioritizing their adoption as the highest-leverage move for AI.
+• Discussion moved to AI-driven automated decision-making, with nutriglow10 calling it currently overhyped but important in five years, and nutriglow4 warning it can widen gaps rather than close them.
+• nutriglow7 expressed concern that automated decision-making benefits only a few players, while nutriglow8 noted industry leaders see it as central to competitiveness.
+• nutriglow10 suggested piloting automated decision-making on a smaller scale before broader rollout.
+• The conversation concluded with discussion on the push for AI regulation, with nutriglow4 noting it is reshaping AI faster than most realize, and nutriglow8 cautioning that regulation could move faster than AI can adapt.</t>
+  </si>
+  <si>
+    <t>2026-08-14T07:39:50.799Z</t>
+  </si>
+  <si>
+    <t>10 User High Volume Discussion 1786692972129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary:
+• Aug 14, 2026 — nutriglow1 opened a discussion asking how the rise of large language models (LLMs) will change AI over the next few years.
+• nutriglow2 noted that LLMs will have real impact but that AI still needs structural reforms alongside them.
+• nutriglow5 offered a contrasting view, suggesting LLMs are not as central to AI as commonly assumed.
+• nutriglow6 warned that LLMs could backfire if AI isn't ready, and nutriglow9 raised concerns about insufficient oversight in LLM adoption.
+• nutriglow10 noted LLMs are already a major planning consideration for organizations, while nutriglow2 recommended investing more in LLMs before AI outgrows our ability to manage it.
+• nutriglow5 shifted the discussion to generative AI coding assistants, asking about their adoption within AI.
+• nutriglow7 called it the biggest recent shift in AI, while nutriglow9 pushed back, saying it hasn't made much difference.
+• nutriglow3 worried adoption of coding assistants may outpace necessary safeguards, and nutriglow6 suggested prioritizing it as the highest-leverage move for AI.
+• nutriglow9 raised whether AI-driven automated decision-making is solving problems or adding complexity.
+• nutriglow10 called it currently overhyped but significant in five years; nutriglow4 cautioned it can widen gaps rather than close them.
+• nutriglow7 expressed concern that automated decision-making benefits only a few players, while nutriglow10 suggested piloting it on a smaller scale before broader rollout.
+• nutriglow3 asked about the push for AI regulation, with nutriglow4 noting it is reshaping AI faster than most realize.
+• nutriglow8 warned that regulation could move faster than AI can adapt, while nutriglow9 noted that organizations focused on regulation are already ahead.</t>
   </si>
 </sst>
 </file>
@@ -139,11 +246,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -484,7 +594,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -614,6 +724,91 @@
         <v>27</v>
       </c>
     </row>
+    <row r="9" ht="409.6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>500</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" ht="210" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>50</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" ht="195" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11">
+        <v>50</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" ht="180" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12">
+        <v>50</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" ht="210" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13">
+        <v>50</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>